<commit_message>
feat: add levels and excel system, and refactor classes
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,22 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>236</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -516,16 +516,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C4" t="n">
-        <v>218</v>
+        <v>1952</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -552,6 +552,87 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>&amp; C:/Python314/python.exe "c:/Users/mortrpestl/Desktop/Archives/mortrpestl/The UPper Hand/1st Year/1st Sem/CS11/cs11project/cs11-project-jugemu-jugemu/Bonus/MainMenu.py"</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>abgs</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ih ang bangis</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: add error codes and fixed waiting times after win/loss
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -516,16 +516,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>1952</v>
+        <v>2272</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
feat: add Flash item and integrate with game
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>total_times</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>total_seconds_played</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,6 +486,7 @@
           <t>11</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,6 +514,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -516,16 +523,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C4" t="n">
-        <v>2272</v>
+        <v>2676</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>45</v>
+      </c>
+      <c r="F4" t="n">
+        <v>241</v>
       </c>
     </row>
     <row r="5">
@@ -554,6 +564,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -581,6 +592,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -608,6 +620,7 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -633,6 +646,99 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: edit item name display and default open directory
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -523,19 +523,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C4" t="n">
-        <v>2676</v>
+        <v>2893</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F4" t="n">
-        <v>241</v>
+        <v>616</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
feat: change behaviour of main menu file
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,6 +593,33 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>{"1": 3.293201446533203, "2": 8.402142763137817, "3": 23.54263138771057, "4": 41.22413158416748, "6": 58.78960871696472}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: animation timings and sound syntax
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,6 +593,48 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>1eNh3mX/t/iNC b0PbK7FD niD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GUEST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>/9P.G</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>p"</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>AsxOEhJ/KYYhH/YpQK</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: UI improvements (level, folder select)
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,6 +719,38 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>DekqsJh8Bk9/2iFQs0Q/JHHXs3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Franz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>kGD"A</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>{}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: add new levels
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -651,32 +651,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>aK</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ahQ</t>
+          <t>Do"B</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Dh</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Db</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DDJcaaor68"bBlHOo"</t>
+          <t>CVrcVaV"THCoQl8Rh</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>liXX88S8l8nT2O8RV"RtTh2OxY4kTyCi{fVa "68goXs8CXssH R8qwhTkMs:Xoga"D2O8 KQTaTcTfzDshqr,DQcHTVeRKaTJs7DoB9</t>
+          <t>liXX88S8l8nT2O8RV"RtTh2OxY4kTyCi{fVa "68goXs8CXssH R8qwhTkMs:Xoga"D2O8 KQTaTcTfzDshqr,DQcHTVeRKaTJs7DoBZs8hUTzG4sT/Cb2gxRheBa hsgwY4kTyOi{fwR Bb7CuQtV VJgx XTfzDsBqr,b"cVDTrt7gb26KTcQt.,isXF8S8BVnhJsV"hsRHOuBt7Y4kTyTi{fx  JgwgVes8"K2s7Y4kTy"i{f7O sg7OoXBa"oQbK"TR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: item logic, levels list
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -651,32 +651,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>aK</t>
+          <t>:D</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Do"B</t>
+          <t>Ch2s</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dh</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Db</t>
+          <t>DD</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CVrcVaV"THCoQl8Rh</t>
+          <t>DVogwTT2RxObBBVOX2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>liXX88S8l8nT2O8RV"RtTh2OxY4kTyCi{fVa "68goXs8CXssH R8qwhTkMs:Xoga"D2O8 KQTaTcTfzDshqr,DQcHTVeRKaTJs7DoBZs8hUTzG4sT/Cb2gxRheBa hsgwY4kTyOi{fwR Bb7CuQtV VJgx XTfzDsBqr,b"cVDTrt7gb26KTcQt.,isXF8S8BVnhJsV"hsRHOuBt7Y4kTyTi{fx  JgwgVes8"K2s7Y4kTy"i{f7O sg7OoXBa"oQbK"TR</t>
+          <t>liXX88S8l8nT2O8RV"RtTh2OxY4kTyCi{fVa "68goXs8CXssH R8qwhTkMs:Xoga"D2O8 KQTaTcTfzDshqr,DQcHTVeRKaTJs7DoBZs8hUTzG4sT/Cb2gxRheBa hsgwY4kTyOi{fwR Bb7CuQtV VJgx XTfzDsBqr,b"cVDTrt7gb26KTcQt.,isXF8S8BVnhJsV"hsRHOuBt7Y4kTyTi{fx  JgwgVes8"K2s7Y4kTy"i{f7O sg7OoXBa"oQbK"TTfzCshqr,D2ctDuhl8:hXlaahXZs8KUtzG4Bs/CbB6wDb"6K cXg{</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: PlayerData (and bee behavior tweak)
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Che</t>
+          <t>OcB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t> </t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>"To6FCohTwgDXgwgV</t>
+          <t>RVoTw:Vhlx:brBVT</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXK8S8TxnDrBtTuhRaRursF:R8qwhVkMs:cotHRo2bwgbssK:TR</t>
+          <t>lisXK8S8TxnDrBtTuhRaRursF:R8qwhVkMs:cotHRo2bwgbssK:TTfzOsQqr,KBc8TThs8"bQ6Kaosb.,isXw8S8TKnDeRw K2stgDXsx Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: Log, Ice, Flash
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OcB</t>
+          <t>aTs</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>:</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>T</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>RVoTw:Vhlx:brBVT</t>
+          <t>aKoswCbBbagb2b7TV</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXK8S8TxnDrBtTuhRaRursF:R8qwhVkMs:cotHRo2bwgbssK:TTfzOsQqr,KBc8TThs8"bQ6Kaosb.,isXw8S8TKnDeRw K2stgDXsx Y</t>
+          <t>lisXK8S8TxnDrBtTuhRaRursF:R8qwhVkMs:cotHRo2bwgbssK:TTfzOsQqr,KBc8TThs8"bQ6Kaosb.,isXw8S8TKnDeRw K2stgDXsx R8qwhokMsaKoswCbBbagb2b7TVR</t>
         </is>
       </c>
     </row>
@@ -551,6 +551,48 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>g5Pan6Zf//ualQAc/6EeeRlFkYd</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>anonymous</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>r2d2c.dvJ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>H:</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>QekQQxR:e0QQRR:Q</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>iG/ZeGoW/QkQQxR:e0QQRR:QC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: sync repos, add colorama, and possible levels
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -1,72 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\cs11-project-si-legends\Bonus\Statistics\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB75EF0-0F13-4C2C-BD75-BF2B365597C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="14370" yWindow="750" windowWidth="14385" windowHeight="14685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>username</t>
-  </si>
-  <si>
-    <t>encrypted_username</t>
-  </si>
-  <si>
-    <t>total_mushrooms_collected</t>
-  </si>
-  <si>
-    <t>total_tiles_walked</t>
-  </si>
-  <si>
-    <t>total_wins</t>
-  </si>
-  <si>
-    <t>total_times</t>
-  </si>
-  <si>
-    <t>total_seconds_played</t>
-  </si>
-  <si>
-    <t>completed_data</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -81,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -405,34 +420,96 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>encrypted_username</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_mushrooms_collected</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_tiles_walked</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>total_wins</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>total_times</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_seconds_played</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>completed_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GUEST</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x/No</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dus</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RKXg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cb</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CX</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> hrc8OKBtaTosRFOD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>lisXw8S8TVno"6xDDXTa:usO7Y4kTyCi{fFC "gtaoBgxDhXswRR8qwhbkMsDVoTKRT"tVOhsBt:cXZs8hUOzG4r6/:o2RF"oeOH:DsO.,isX88S8ltnXQ6HDhrlw"bJRa R8qwhDkMs"DoBa:u2baObJO7 R8qwhokMsOXoOHObstVRXXbaOXTfzDs2qr,ohcKauelH:KssaOoBZs8hUgzG4XO/achlxTDsR8:h2g.,iQXw8S8Ttg rT7aVhbaDTelVY4k6yOi{f7" sbFDuQt8:KQbHRR8qVhTkMs ToTVRVrO7OT2gt cTfzCsBqr,cecwDK2OKCoBsFghJZs8KURzG4rR/guQg7Cu2tV:DsT.,iQXx8S8Twg egx"bslwCchTtRR8qVhVkMsCuostCcesV"chlagb2Zs8bU6zG4rt/CKeB7:oBt8"VJBHY4klyOi{fV" JOwRcXOwgcB6aTR8qKhTkMsCuoB8"ueTtDDhTHTKTfzOsBqr,KQctCTrRVgX"67"oBR.,irXH8S8RFnbQtVDKXBx:b"B.,irXF8S8O7nX2tagbs6tgTebaRR8qKhhkMsCbhcK DsbFaDQg7CcR</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add BGM systems
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dus</t>
+          <t>DbB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RKXg</t>
+          <t>ah2b</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cb</t>
+          <t>CX</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CX</t>
+          <t>OD</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> hrc8OKBtaTosRFOD</t>
+          <t>CVos8OVestgbXlKCK2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXw8S8TVno"6xDDXTa:usO7Y4kTyCi{fFC "gtaoBgxDhXswRR8qwhbkMsDVoTKRT"tVOhsBt:cXZs8hUOzG4r6/:o2RF"oeOH:DsO.,isX88S8ltnXQ6HDhrlw"bJRa R8qwhDkMs"DoBa:u2baObJO7 R8qwhokMsOXoOHObstVRXXbaOXTfzDs2qr,ohcKauelH:KssaOoBZs8hUgzG4XO/achlxTDsR8:h2g.,iQXw8S8Ttg rT7aVhbaDTelVY4k6yOi{f7" sbFDuQt8:KQbHRR8qVhTkMs ToTVRVrO7OT2gt cTfzCsBqr,cecwDK2OKCoBsFghJZs8KURzG4rR/guQg7Cu2tV:DsT.,iQXx8S8Twg egx"bslwCchTtRR8qVhVkMsCuostCcesV"chlagb2Zs8bU6zG4rt/CKeB7:oBt8"VJBHY4klyOi{fV" JOwRcXOwgcB6aTR8qKhTkMsCuoB8"ueTtDDhTHTKTfzOsBqr,KQctCTrRVgX"67"oBR.,irXH8S8RFnbQtVDKXBx:b"B.,irXF8S8O7nX2tagbs6tgTebaRR8qKhhkMsCbhcK DsbFaDQg7CcR</t>
+          <t>lisXw8S8TVno"6xDDXTa:usO7Y4kTyCi{fFC "gtaoBgxDhXswRR8qwhbkMsDVoTKRT"tVOhsBt:cXZs8hUOzG4r6/:o2RF"oeOH:DsO.,isX88S8ltnXQ6HDhrlw"bJRa R8qwhDkMs"DoBa:u2baObJO7 R8qwhokMsOXoOHObstVRXXbaOXTfzDs2qr,ohcKauelH:KssaOoBZs8hUgzG4XO/achlxTDsR8:h2g.,iQXw8S8Ttg rT7aVhbaDTelVY4k6yOi{f7" sbFDuQt8:KQbHRR8qVhTkMs ToTVRVrO7OT2gt cTfzCsBqr,T2c7OhssFgTX6w"V"Zs8KURzG4rs/OuebxTuhT8CbXlxY4k6yTi{fwDuosaTVrTKDKBRwgTTfzCsJqr,KectgKBstCVBRK"urb.,irXV8S8l8nKQsFRD"t8aVJgF:R8qKhbkMsCVog7DTBO7DuBtV"XTfzOsXqr,KecFaVeswghhRw:XQZs8bUtzG4Q6/gKXlHCu2BVRV"tHY4kly:i{fH  r68ChQOFTDrBFY4kly i{f7R 2b8"urTVguXsx"TTfzOssqr,KrR/OohTx ch6aRKBZs8KU6zG4sTxnbeRx ohTKgD"RKy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: sound cache, level loading screen
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DbB</t>
+          <t>Dch</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ah2b</t>
+          <t>:uXO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CX</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>OD</t>
+          <t>Rb</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CVos8OVestgbXlKCK2</t>
+          <t>CootVRXhBtao2stCVr</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXw8S8TVno"6xDDXTa:usO7Y4kTyCi{fFC "gtaoBgxDhXswRR8qwhbkMsDVoTKRT"tVOhsBt:cXZs8hUOzG4r6/:o2RF"oeOH:DsO.,isX88S8ltnXQ6HDhrlw"bJRa R8qwhDkMs"DoBa:u2baObJO7 R8qwhokMsOXoOHObstVRXXbaOXTfzDs2qr,ohcKauelH:KssaOoBZs8hUgzG4XO/achlxTDsR8:h2g.,iQXw8S8Ttg rT7aVhbaDTelVY4k6yOi{f7" sbFDuQt8:KQbHRR8qVhTkMs ToTVRVrO7OT2gt cTfzCsBqr,T2c7OhssFgTX6w"V"Zs8KURzG4rs/OuebxTuhT8CbXlxY4k6yTi{fwDuosaTVrTKDKBRwgTTfzCsJqr,KectgKBstCVBRK"urb.,irXV8S8l8nKQsFRD"t8aVJgF:R8qKhbkMsCVog7DTBO7DuBtV"XTfzOsXqr,KecFaVeswghhRw:XQZs8bUtzG4Q6/gKXlHCu2BVRV"tHY4kly:i{fH  r68ChQOFTDrBFY4kly i{f7R 2b8"urTVguXsx"TTfzOssqr,KrR/OohTx ch6aRKBZs8KU6zG4sTxnbeRx ohTKgD"RKy</t>
+          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMs KoBagc"taThsOtDTTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,VhcF"Debx"brg7RoTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,oXcwCTJl7RbXbagoBZs8KUtzG4Xb/RbsTt uXOVDVJB.,iQXH8S868nursVgbss7ghJTHaR8qVhXkMsDhect"XJlwOhQtHDuXZs8KUgzG4Qs/guQttgKJtHOVelxY4klyCi{fKa Q6t ThB8acJga DTfzOsrqr,K"cw VJOxgVstt:VBb.,irX78S86tnoBgtgheTH:hhbVY4klyai{fVC e67ODQsx KXgFaDTfzOshqr,D"cKCcQTVRo2RK oTfzOs"qr,TXcxTcJsKDKes7gXJO.,irXw8S86K: rBHDX"tHCVX68Y4k6yCi{fwDXolt:X"BHDbeRF:bTfzCs"qr,Vec8"TXTVTurR7"VR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add and adjust more SFX features
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dch</t>
+          <t>CK2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>:uXO</t>
+          <t>TbXg</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>Rc</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rb</t>
+          <t>ao</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CootVRXhBtao2stCVr</t>
+          <t xml:space="preserve"> co6waTXBH:TQRtTD</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMs KoBagc"taThsOtDTTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,VhcF"Debx"brg7RoTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,oXcwCTJl7RbXbagoBZs8KUtzG4Xb/RbsTt uXOVDVJB.,iQXH8S868nursVgbss7ghJTHaR8qVhXkMsDhect"XJlwOhQtHDuXZs8KUgzG4Qs/guQttgKJtHOVelxY4klyCi{fKa Q6t ThB8acJga DTfzOsrqr,K"cw VJOxgVstt:VBb.,irX78S86tnoBgtgheTH:hhbVY4klyai{fVC e67ODQsx KXgFaDTfzOshqr,D"cKCcQTVRo2RK oTfzOs"qr,TXcxTcJsKDKes7gXJO.,irXw8S86K: rBHDX"tHCVX68Y4k6yCi{fwDXolt:X"BHDbeRF:bTfzCs"qr,Vec8"TXTVTurR7"VR</t>
+          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMs KoBagc"taThsOtDTTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJ9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: existing user log-in
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,32 +483,74 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CK2</t>
+          <t>CbB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TbXg</t>
+          <t>TTBb</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rc</t>
+          <t>RX</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ao</t>
+          <t>:h</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> co6waTXBH:TQRtTD</t>
+          <t>DcoOH:bJsK hr6V:bQ</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMs KoBagc"taThsOtDTTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJ9</t>
+          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMsCVo6HaDJOK V2sHaKTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mortr</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fi,bj</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hh</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>H2b</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CecxOpJgtiNBRxF/hl</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6kTyiU{f7l1hTFiN2bFiqhOKF{8qVNqkMsHpobalNJs7O4hbw9qr9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: reduced ruff errors in Main
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -483,32 +483,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CbB</t>
+          <t>Oue</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TTBb</t>
+          <t>"uBt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>RX</t>
+          <t>aK</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>:h</t>
+          <t>:D</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DcoOH:bJsK hr6V:bQ</t>
+          <t>RhoBH:V"RxObrOKauh</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMsCVo6HaDJOK V2sHaKTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJ9</t>
+          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMsCVo6HaDJOK V2sHaKTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJZs8TUTzG4rt/RKeT7guQBa"V2b.,iXX78S8RxnXrOwDo2baRuXl{</t>
         </is>
       </c>
     </row>
@@ -525,32 +525,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hh</t>
+          <t>H"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>H2b</t>
+          <t>"2b</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>"</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>"</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CecxOpJgtiNBRxF/hl</t>
+          <t>CrcHHpXlH/42b8O"B</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>6kTyiU{f7l1hTFiN2bFiqhOKF{8qVNqkMsHpobalNJs7O4hbw9qr9</t>
+          <t>6kTyiU{f7l1hTFiN2bFiqhOKF{8qVNqkMsHpobalNJs7O4hbw9qrZsJ.UTzhhrl//CeOK/qBbxKNQt{</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add level 1, fix bonus
</commit_message>
<xml_diff>
--- a/Bonus/Statistics/PlayerData.xlsx
+++ b/Bonus/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,48 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>6kTyiU{f7l1hTFiN2bFiqhOKF{8qVNqkMsHpobalNJs7O4hbw9qrZsJ.UTzhhrl//CeOK/qBbxKNQt{</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mortrpestl</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLGbGZYCb </t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>uoRt</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>9a9/p7BOKiUa9a9HBO</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>E69ylU{fV/oOpx9.rOx/oE9w9.R</t>
         </is>
       </c>
     </row>

</xml_diff>